<commit_message>
Start English translation ; add 2 Disperse Troops Cards per Deck
</commit_message>
<xml_diff>
--- a/docs/Cartes-Actions-Repartition.xlsx
+++ b/docs/Cartes-Actions-Repartition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Documents\GitHub\Terre-de-Barons\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F3EFA22-DF28-479F-9755-4AF62BB31748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55318E12-7E5E-438B-A1F0-213DAD004D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-9120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Présentation" sheetId="2" r:id="rId1"/>
@@ -768,7 +768,7 @@
       <c r="G3" s="19"/>
       <c r="H3" s="14">
         <f>SUM(D3:D15)</f>
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
@@ -817,11 +817,11 @@
       </c>
       <c r="F6" s="10">
         <f>E6+E9</f>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G6" s="13">
         <f>SUM(D6:D11)</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H6" s="15"/>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="E9" s="10">
         <f>SUM(D9:D10)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F9" s="36"/>
       <c r="G9" s="13"/>
@@ -881,7 +881,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E10" s="35"/>
       <c r="F10" s="35"/>

</xml_diff>

<commit_message>
First English translation ; mise en cohérence de la règle française
</commit_message>
<xml_diff>
--- a/docs/Cartes-Actions-Repartition.xlsx
+++ b/docs/Cartes-Actions-Repartition.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Documents\GitHub\Terre-de-Barons\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55318E12-7E5E-438B-A1F0-213DAD004D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78CCFA3E-4123-47F3-A428-7A2290BB0776}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-9120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,24 +50,6 @@
     <t>Chevauchée Lointaine</t>
   </si>
   <si>
-    <t>Déplacer Officier 3+</t>
-  </si>
-  <si>
-    <t>Déplacer Officier 2+</t>
-  </si>
-  <si>
-    <t>Déplacer Officier 1+</t>
-  </si>
-  <si>
-    <t>Recruter Troupes 3+</t>
-  </si>
-  <si>
-    <t>Recruter Troupes 1+</t>
-  </si>
-  <si>
-    <t>Recruter Troupes 2+</t>
-  </si>
-  <si>
     <t>Recruter Chevalier</t>
   </si>
   <si>
@@ -87,6 +69,24 @@
   </si>
   <si>
     <t>Exiler Chevalier</t>
+  </si>
+  <si>
+    <t>Déplacer Seigneur 3</t>
+  </si>
+  <si>
+    <t>Déplacer Seigneur 2</t>
+  </si>
+  <si>
+    <t>Déplacer Seigneur 1</t>
+  </si>
+  <si>
+    <t>Recruter Troupes 3</t>
+  </si>
+  <si>
+    <t>Recruter Troupes 2</t>
+  </si>
+  <si>
+    <t>Recruter Troupes 1</t>
   </si>
 </sst>
 </file>
@@ -735,16 +735,16 @@
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F2" s="7"/>
       <c r="G2" s="8"/>
@@ -752,7 +752,7 @@
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C3" s="1">
         <v>3</v>
@@ -773,7 +773,7 @@
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1">
         <v>2</v>
@@ -788,7 +788,7 @@
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1">
         <v>1</v>
@@ -803,7 +803,7 @@
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C6" s="2">
         <v>3</v>
@@ -827,7 +827,7 @@
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C7" s="2">
         <v>2</v>
@@ -842,7 +842,7 @@
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C8" s="2">
         <v>1</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C11" s="2">
         <v>3</v>
@@ -929,7 +929,7 @@
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C13" s="1">
         <v>3</v>
@@ -944,7 +944,7 @@
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C14" s="1">
         <v>3</v>
@@ -959,7 +959,7 @@
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C15" s="5">
         <v>3</v>

</xml_diff>

<commit_message>
Mise à jour des règles avec Hérauts de Pourparlers - en français
</commit_message>
<xml_diff>
--- a/docs/Cartes-Actions-Repartition.xlsx
+++ b/docs/Cartes-Actions-Repartition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Documents\GitHub\Terre-de-Barons\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F25D181A-2E74-4FF6-BAB6-B7658685AD3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C16ADF56-A970-4969-8392-0C077EF94F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-9120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-9120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards-fr" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
   <si>
     <t>Nombre</t>
   </si>
@@ -411,6 +411,28 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -428,9 +450,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -498,25 +517,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -808,16 +808,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1E300F5-BB8C-42D4-B150-781935673603}">
-  <dimension ref="B2:H15"/>
+  <dimension ref="B2:K15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" customWidth="1"/>
     <col min="2" max="2" width="23.7109375" customWidth="1"/>
     <col min="3" max="4" width="7.7109375" customWidth="1"/>
     <col min="5" max="8" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
@@ -827,14 +829,20 @@
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="9"/>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F2" s="15"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="17"/>
+      <c r="J2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
@@ -844,18 +852,24 @@
       <c r="D3" s="1">
         <v>4</v>
       </c>
-      <c r="E3" s="17">
+      <c r="E3" s="24">
         <f>SUM(D3:D5)</f>
         <v>15</v>
       </c>
-      <c r="F3" s="18"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="14">
+      <c r="F3" s="25"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="21">
         <f>SUM(D3:D15)</f>
         <v>42</v>
       </c>
-    </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K3" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>12</v>
       </c>
@@ -865,12 +879,18 @@
       <c r="D4" s="1">
         <v>5</v>
       </c>
-      <c r="E4" s="20"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="15"/>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E4" s="27"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="22"/>
+      <c r="J4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>13</v>
       </c>
@@ -880,12 +900,18 @@
       <c r="D5" s="1">
         <v>6</v>
       </c>
-      <c r="E5" s="23"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="15"/>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E5" s="30"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="22"/>
+      <c r="J5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>14</v>
       </c>
@@ -895,21 +921,27 @@
       <c r="D6" s="2">
         <v>2</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="18">
         <f>SUM(D6:D8)</f>
         <v>9</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="18">
         <f>E6+E9</f>
         <v>17</v>
       </c>
-      <c r="G6" s="13">
+      <c r="G6" s="11">
         <f>SUM(D6:D11)</f>
         <v>23</v>
       </c>
-      <c r="H6" s="15"/>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="H6" s="22"/>
+      <c r="J6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>15</v>
       </c>
@@ -919,12 +951,18 @@
       <c r="D7" s="2">
         <v>3</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="15"/>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E7" s="19"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="22"/>
+      <c r="J7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K7" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>16</v>
       </c>
@@ -934,12 +972,18 @@
       <c r="D8" s="2">
         <v>4</v>
       </c>
-      <c r="E8" s="12"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="15"/>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E8" s="20"/>
+      <c r="F8" s="43"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="22"/>
+      <c r="J8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>2</v>
       </c>
@@ -949,15 +993,21 @@
       <c r="D9" s="2">
         <v>3</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="18">
         <f>SUM(D9:D10)</f>
         <v>8</v>
       </c>
-      <c r="F9" s="36"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="15"/>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F9" s="43"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="22"/>
+      <c r="J9" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K9" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>1</v>
       </c>
@@ -967,12 +1017,18 @@
       <c r="D10" s="2">
         <v>5</v>
       </c>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="15"/>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E10" s="42"/>
+      <c r="F10" s="42"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="22"/>
+      <c r="J10" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K10" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
         <v>6</v>
       </c>
@@ -990,10 +1046,16 @@
         <f>E11</f>
         <v>6</v>
       </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="15"/>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="G11" s="11"/>
+      <c r="H11" s="22"/>
+      <c r="J11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K11" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>3</v>
       </c>
@@ -1003,15 +1065,21 @@
       <c r="D12" s="1">
         <v>1</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="33">
         <f>SUM(D12:D15)</f>
         <v>4</v>
       </c>
-      <c r="F12" s="27"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="15"/>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F12" s="34"/>
+      <c r="G12" s="35"/>
+      <c r="H12" s="22"/>
+      <c r="J12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K12" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>4</v>
       </c>
@@ -1021,12 +1089,18 @@
       <c r="D13" s="1">
         <v>1</v>
       </c>
-      <c r="E13" s="29"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="15"/>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E13" s="36"/>
+      <c r="F13" s="37"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="22"/>
+      <c r="J13" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K13" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>10</v>
       </c>
@@ -1036,12 +1110,18 @@
       <c r="D14" s="1">
         <v>1</v>
       </c>
-      <c r="E14" s="29"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="15"/>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E14" s="36"/>
+      <c r="F14" s="37"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="22"/>
+      <c r="J14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K14" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
         <v>7</v>
       </c>
@@ -1051,10 +1131,16 @@
       <c r="D15" s="1">
         <v>1</v>
       </c>
-      <c r="E15" s="32"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="16"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="40"/>
+      <c r="G15" s="41"/>
+      <c r="H15" s="23"/>
+      <c r="J15" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K15" s="1">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1068,7 +1154,7 @@
     <mergeCell ref="F6:F10"/>
   </mergeCells>
   <conditionalFormatting sqref="D3:D5">
-    <cfRule type="colorScale" priority="25">
+    <cfRule type="colorScale" priority="38">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1080,7 +1166,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D3:D8 D12:D15">
-    <cfRule type="colorScale" priority="18">
+    <cfRule type="colorScale" priority="31">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1088,7 +1174,7 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="19">
+    <cfRule type="colorScale" priority="32">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1100,7 +1186,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D3:D15">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1110,7 +1196,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6:D8">
-    <cfRule type="colorScale" priority="24">
+    <cfRule type="colorScale" priority="37">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1122,7 +1208,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9">
-    <cfRule type="colorScale" priority="8">
+    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1134,7 +1220,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9:D10">
-    <cfRule type="colorScale" priority="5">
+    <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1142,7 +1228,7 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="6">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1154,7 +1240,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D10">
-    <cfRule type="colorScale" priority="7">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1166,7 +1252,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D11">
-    <cfRule type="colorScale" priority="2">
+    <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1174,6 +1260,146 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D12:D15">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:K5">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:K8 K12:K15">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:K15">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K6:K8">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K9">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K9:K10">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K10">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -1195,8 +1421,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D12:D15">
-    <cfRule type="colorScale" priority="20">
+  <conditionalFormatting sqref="K12:K15">
+    <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1228,21 +1454,21 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="37" t="s">
+      <c r="D2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="38" t="s">
+      <c r="E2" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
@@ -1254,13 +1480,13 @@
       <c r="D3" s="1">
         <v>4</v>
       </c>
-      <c r="E3" s="40">
+      <c r="E3" s="9">
         <f>SUM(D3:D5)</f>
         <v>15</v>
       </c>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="41">
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="10">
         <f>SUM(D3:D15)</f>
         <v>42</v>
       </c>
@@ -1275,10 +1501,10 @@
       <c r="D4" s="1">
         <v>5</v>
       </c>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="41"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="10"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
@@ -1290,10 +1516,10 @@
       <c r="D5" s="1">
         <v>6</v>
       </c>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="41"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="10"/>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
@@ -1305,19 +1531,19 @@
       <c r="D6" s="2">
         <v>2</v>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="11">
         <f>SUM(D6:D8)</f>
         <v>9</v>
       </c>
-      <c r="F6" s="13">
+      <c r="F6" s="11">
         <f>E6+E9</f>
         <v>17</v>
       </c>
-      <c r="G6" s="13">
+      <c r="G6" s="11">
         <f>SUM(D6:D11)</f>
         <v>23</v>
       </c>
-      <c r="H6" s="41"/>
+      <c r="H6" s="10"/>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
@@ -1329,10 +1555,10 @@
       <c r="D7" s="2">
         <v>3</v>
       </c>
-      <c r="E7" s="13"/>
-      <c r="F7" s="42"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="41"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="10"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
@@ -1344,10 +1570,10 @@
       <c r="D8" s="2">
         <v>4</v>
       </c>
-      <c r="E8" s="13"/>
-      <c r="F8" s="42"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="41"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="10"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
@@ -1359,13 +1585,13 @@
       <c r="D9" s="2">
         <v>3</v>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="11">
         <f>SUM(D9:D10)</f>
         <v>8</v>
       </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="41"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="10"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
@@ -1377,10 +1603,10 @@
       <c r="D10" s="2">
         <v>5</v>
       </c>
-      <c r="E10" s="42"/>
-      <c r="F10" s="42"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="41"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="10"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
@@ -1400,8 +1626,8 @@
         <f>E11</f>
         <v>6</v>
       </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="41"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="10"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
@@ -1413,13 +1639,13 @@
       <c r="D12" s="1">
         <v>1</v>
       </c>
-      <c r="E12" s="43">
+      <c r="E12" s="13">
         <f>SUM(D12:D15)</f>
         <v>4</v>
       </c>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="41"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="10"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
@@ -1431,10 +1657,10 @@
       <c r="D13" s="1">
         <v>1</v>
       </c>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="41"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="10"/>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
@@ -1446,10 +1672,10 @@
       <c r="D14" s="1">
         <v>1</v>
       </c>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="41"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="10"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
@@ -1461,10 +1687,10 @@
       <c r="D15" s="1">
         <v>1</v>
       </c>
-      <c r="E15" s="43"/>
-      <c r="F15" s="43"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="41"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>

<commit_message>
Première réécriture avec Espion et nouveau second deck
</commit_message>
<xml_diff>
--- a/docs/Cartes-Actions-Repartition.xlsx
+++ b/docs/Cartes-Actions-Repartition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Documents\GitHub\Terre-de-Barons\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C16ADF56-A970-4969-8392-0C077EF94F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3037AD7E-3FC7-4300-9229-51FB02E80542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-9120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards-fr" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="36">
   <si>
     <t>Nombre</t>
   </si>
@@ -139,6 +139,12 @@
   </si>
   <si>
     <t>Court Intrigue</t>
+  </si>
+  <si>
+    <t>Espion</t>
+  </si>
+  <si>
+    <t>Spy</t>
   </si>
 </sst>
 </file>
@@ -394,7 +400,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -414,23 +420,7 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -450,15 +440,15 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -498,27 +488,44 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -808,7 +815,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1E300F5-BB8C-42D4-B150-781935673603}">
-  <dimension ref="B2:K15"/>
+  <dimension ref="B2:K16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" customWidth="1"/>
@@ -829,12 +836,12 @@
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="15"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="17"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="11"/>
       <c r="J2" s="3" t="s">
         <v>8</v>
       </c>
@@ -852,15 +859,15 @@
       <c r="D3" s="1">
         <v>4</v>
       </c>
-      <c r="E3" s="24">
+      <c r="E3" s="18">
         <f>SUM(D3:D5)</f>
         <v>15</v>
       </c>
-      <c r="F3" s="25"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="21">
-        <f>SUM(D3:D15)</f>
-        <v>42</v>
+      <c r="F3" s="19"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="16">
+        <f>SUM(D3:D16)</f>
+        <v>43</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>11</v>
@@ -879,10 +886,10 @@
       <c r="D4" s="1">
         <v>5</v>
       </c>
-      <c r="E4" s="27"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="22"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="17"/>
       <c r="J4" s="1" t="s">
         <v>12</v>
       </c>
@@ -900,10 +907,10 @@
       <c r="D5" s="1">
         <v>6</v>
       </c>
-      <c r="E5" s="30"/>
-      <c r="F5" s="31"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="22"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="17"/>
       <c r="J5" s="1" t="s">
         <v>13</v>
       </c>
@@ -921,19 +928,19 @@
       <c r="D6" s="2">
         <v>2</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="12">
         <f>SUM(D6:D8)</f>
         <v>9</v>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="12">
         <f>E6+E9</f>
         <v>17</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="15">
         <f>SUM(D6:D11)</f>
         <v>23</v>
       </c>
-      <c r="H6" s="22"/>
+      <c r="H6" s="17"/>
       <c r="J6" s="2" t="s">
         <v>14</v>
       </c>
@@ -951,10 +958,10 @@
       <c r="D7" s="2">
         <v>3</v>
       </c>
-      <c r="E7" s="19"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="22"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="17"/>
       <c r="J7" s="2" t="s">
         <v>15</v>
       </c>
@@ -972,10 +979,10 @@
       <c r="D8" s="2">
         <v>4</v>
       </c>
-      <c r="E8" s="20"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="22"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="17"/>
       <c r="J8" s="2" t="s">
         <v>16</v>
       </c>
@@ -993,13 +1000,13 @@
       <c r="D9" s="2">
         <v>3</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="12">
         <f>SUM(D9:D10)</f>
         <v>8</v>
       </c>
-      <c r="F9" s="43"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="22"/>
+      <c r="F9" s="33"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="17"/>
       <c r="J9" s="2" t="s">
         <v>2</v>
       </c>
@@ -1017,10 +1024,10 @@
       <c r="D10" s="2">
         <v>5</v>
       </c>
-      <c r="E10" s="42"/>
-      <c r="F10" s="42"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="22"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="17"/>
       <c r="J10" s="2" t="s">
         <v>1</v>
       </c>
@@ -1038,16 +1045,16 @@
       <c r="D11" s="2">
         <v>6</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="7">
         <f>D11</f>
         <v>6</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="7">
         <f>E11</f>
         <v>6</v>
       </c>
-      <c r="G11" s="11"/>
-      <c r="H11" s="22"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="17"/>
       <c r="J11" s="2" t="s">
         <v>6</v>
       </c>
@@ -1062,16 +1069,16 @@
       <c r="C12" s="1">
         <v>3</v>
       </c>
-      <c r="D12" s="1">
-        <v>1</v>
-      </c>
-      <c r="E12" s="33">
-        <f>SUM(D12:D15)</f>
-        <v>4</v>
-      </c>
-      <c r="F12" s="34"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="22"/>
+      <c r="D12" s="38">
+        <v>1</v>
+      </c>
+      <c r="E12" s="27">
+        <f>SUM(D12:D16)</f>
+        <v>5</v>
+      </c>
+      <c r="F12" s="28"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="17"/>
       <c r="J12" s="1" t="s">
         <v>3</v>
       </c>
@@ -1086,13 +1093,13 @@
       <c r="C13" s="1">
         <v>3</v>
       </c>
-      <c r="D13" s="1">
-        <v>1</v>
-      </c>
-      <c r="E13" s="36"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="38"/>
-      <c r="H13" s="22"/>
+      <c r="D13" s="38">
+        <v>1</v>
+      </c>
+      <c r="E13" s="30"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="17"/>
       <c r="J13" s="1" t="s">
         <v>4</v>
       </c>
@@ -1107,13 +1114,13 @@
       <c r="C14" s="1">
         <v>3</v>
       </c>
-      <c r="D14" s="1">
-        <v>1</v>
-      </c>
-      <c r="E14" s="36"/>
-      <c r="F14" s="37"/>
-      <c r="G14" s="38"/>
-      <c r="H14" s="22"/>
+      <c r="D14" s="38">
+        <v>1</v>
+      </c>
+      <c r="E14" s="30"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="17"/>
       <c r="J14" s="1" t="s">
         <v>10</v>
       </c>
@@ -1128,17 +1135,38 @@
       <c r="C15" s="5">
         <v>3</v>
       </c>
-      <c r="D15" s="1">
-        <v>1</v>
-      </c>
-      <c r="E15" s="39"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="23"/>
+      <c r="D15" s="38">
+        <v>1</v>
+      </c>
+      <c r="E15" s="30"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="17"/>
       <c r="J15" s="5" t="s">
         <v>7</v>
       </c>
       <c r="K15" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B16" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="5">
+        <v>2</v>
+      </c>
+      <c r="D16" s="38">
+        <v>1</v>
+      </c>
+      <c r="E16" s="40"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="43"/>
+      <c r="J16" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K16" s="1">
         <v>1</v>
       </c>
     </row>
@@ -1147,26 +1175,26 @@
     <mergeCell ref="E2:H2"/>
     <mergeCell ref="E6:E8"/>
     <mergeCell ref="G6:G11"/>
-    <mergeCell ref="H3:H15"/>
     <mergeCell ref="E3:G5"/>
-    <mergeCell ref="E12:G15"/>
     <mergeCell ref="E9:E10"/>
     <mergeCell ref="F6:F10"/>
+    <mergeCell ref="E12:G16"/>
+    <mergeCell ref="H3:H16"/>
   </mergeCells>
   <conditionalFormatting sqref="D3:D5">
-    <cfRule type="colorScale" priority="38">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D8 D12:D15">
-    <cfRule type="colorScale" priority="31">
+    <cfRule type="colorScale" priority="40">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3:D8 D12:D16">
+    <cfRule type="colorScale" priority="33">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1174,19 +1202,19 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="32">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D15">
-    <cfRule type="colorScale" priority="14">
+    <cfRule type="colorScale" priority="34">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3:D16">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1196,7 +1224,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6:D8">
-    <cfRule type="colorScale" priority="37">
+    <cfRule type="colorScale" priority="39">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1208,7 +1236,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9">
-    <cfRule type="colorScale" priority="21">
+    <cfRule type="colorScale" priority="23">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1220,7 +1248,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9:D10">
-    <cfRule type="colorScale" priority="18">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1228,7 +1256,7 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="19">
+    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1240,7 +1268,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D10">
-    <cfRule type="colorScale" priority="20">
+    <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1252,7 +1280,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D11">
-    <cfRule type="colorScale" priority="15">
+    <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1260,29 +1288,29 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D12:D15">
-    <cfRule type="colorScale" priority="33">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D12:D16">
+    <cfRule type="colorScale" priority="35">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1294,19 +1322,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K3:K5">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K3:K8 K12:K15">
-    <cfRule type="colorScale" priority="9">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:K8 K12:K16">
+    <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1314,18 +1342,18 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K3:K15">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:K16">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1336,7 +1364,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6:K8">
-    <cfRule type="colorScale" priority="12">
+    <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1348,7 +1376,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K9">
-    <cfRule type="colorScale" priority="8">
+    <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1360,7 +1388,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K9:K10">
-    <cfRule type="colorScale" priority="5">
+    <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1368,7 +1396,7 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="6">
+    <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1380,7 +1408,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K10">
-    <cfRule type="colorScale" priority="7">
+    <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1392,7 +1420,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="colorScale" priority="2">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1400,29 +1428,29 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K12:K15">
-    <cfRule type="colorScale" priority="11">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12:K16">
+    <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1436,14 +1464,14 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="G6 E12 E3 E9 E6" formulaRange="1"/>
+    <ignoredError sqref="G6 E3 E9 E6 E12" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{592FDED2-945D-4571-B170-2CC455B62199}">
-  <dimension ref="B2:H15"/>
+  <dimension ref="B2:K16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" customWidth="1"/>
@@ -1451,9 +1479,10 @@
     <col min="3" max="3" width="7.7109375" customWidth="1"/>
     <col min="4" max="4" width="8.42578125" customWidth="1"/>
     <col min="5" max="8" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
         <v>17</v>
       </c>
@@ -1463,14 +1492,20 @@
       <c r="D2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="J2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>21</v>
       </c>
@@ -1480,18 +1515,24 @@
       <c r="D3" s="1">
         <v>4</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="36">
         <f>SUM(D3:D5)</f>
         <v>15</v>
       </c>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="10">
-        <f>SUM(D3:D15)</f>
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="16">
+        <f>SUM(D3:D16)</f>
+        <v>43</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>22</v>
       </c>
@@ -1501,12 +1542,18 @@
       <c r="D4" s="1">
         <v>5</v>
       </c>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="10"/>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="17"/>
+      <c r="J4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>23</v>
       </c>
@@ -1516,12 +1563,18 @@
       <c r="D5" s="1">
         <v>6</v>
       </c>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="10"/>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="17"/>
+      <c r="J5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K5" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>24</v>
       </c>
@@ -1531,21 +1584,27 @@
       <c r="D6" s="2">
         <v>2</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="15">
         <f>SUM(D6:D8)</f>
         <v>9</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="15">
         <f>E6+E9</f>
         <v>17</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="15">
         <f>SUM(D6:D11)</f>
         <v>23</v>
       </c>
-      <c r="H6" s="10"/>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="H6" s="17"/>
+      <c r="J6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>25</v>
       </c>
@@ -1555,12 +1614,18 @@
       <c r="D7" s="2">
         <v>3</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="10"/>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E7" s="15"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="17"/>
+      <c r="J7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K7" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>26</v>
       </c>
@@ -1570,12 +1635,18 @@
       <c r="D8" s="2">
         <v>4</v>
       </c>
-      <c r="E8" s="11"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="10"/>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E8" s="15"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="17"/>
+      <c r="J8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K8" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>27</v>
       </c>
@@ -1585,15 +1656,21 @@
       <c r="D9" s="2">
         <v>3</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="15">
         <f>SUM(D9:D10)</f>
         <v>8</v>
       </c>
-      <c r="F9" s="12"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="10"/>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F9" s="37"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="17"/>
+      <c r="J9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K9" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>28</v>
       </c>
@@ -1603,12 +1680,18 @@
       <c r="D10" s="2">
         <v>5</v>
       </c>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="10"/>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E10" s="37"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="17"/>
+      <c r="J10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K10" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
         <v>29</v>
       </c>
@@ -1626,10 +1709,16 @@
         <f>E11</f>
         <v>6</v>
       </c>
-      <c r="G11" s="11"/>
-      <c r="H11" s="10"/>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="G11" s="15"/>
+      <c r="H11" s="17"/>
+      <c r="J11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K11" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>30</v>
       </c>
@@ -1639,15 +1728,21 @@
       <c r="D12" s="1">
         <v>1</v>
       </c>
-      <c r="E12" s="13">
-        <f>SUM(D12:D15)</f>
-        <v>4</v>
-      </c>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="10"/>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E12" s="27">
+        <f>SUM(D12:D16)</f>
+        <v>5</v>
+      </c>
+      <c r="F12" s="28"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="17"/>
+      <c r="J12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K12" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>31</v>
       </c>
@@ -1657,12 +1752,18 @@
       <c r="D13" s="1">
         <v>1</v>
       </c>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="10"/>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E13" s="30"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="17"/>
+      <c r="J13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K13" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>32</v>
       </c>
@@ -1672,12 +1773,18 @@
       <c r="D14" s="1">
         <v>1</v>
       </c>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="10"/>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E14" s="30"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="17"/>
+      <c r="J14" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K14" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
         <v>33</v>
       </c>
@@ -1687,36 +1794,63 @@
       <c r="D15" s="1">
         <v>1</v>
       </c>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="10"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="17"/>
+      <c r="J15" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K15" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B16" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="5">
+        <v>2</v>
+      </c>
+      <c r="D16" s="1">
+        <v>1</v>
+      </c>
+      <c r="E16" s="44"/>
+      <c r="F16" s="45"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="43"/>
+      <c r="J16" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="K16" s="1">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="E2:H2"/>
     <mergeCell ref="E3:G5"/>
-    <mergeCell ref="H3:H15"/>
     <mergeCell ref="E6:E8"/>
     <mergeCell ref="F6:F10"/>
     <mergeCell ref="G6:G11"/>
     <mergeCell ref="E9:E10"/>
-    <mergeCell ref="E12:G15"/>
+    <mergeCell ref="E12:G16"/>
+    <mergeCell ref="H3:H16"/>
   </mergeCells>
   <conditionalFormatting sqref="D3:D5">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D8 D12:D15">
-    <cfRule type="colorScale" priority="9">
+    <cfRule type="colorScale" priority="27">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3:D8 D12:D16">
+    <cfRule type="colorScale" priority="23">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1724,19 +1858,19 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D15">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3:D16">
+    <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1746,7 +1880,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6:D8">
-    <cfRule type="colorScale" priority="12">
+    <cfRule type="colorScale" priority="26">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1758,7 +1892,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9">
-    <cfRule type="colorScale" priority="8">
+    <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1770,7 +1904,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9:D10">
-    <cfRule type="colorScale" priority="5">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1778,7 +1912,7 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="6">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1790,7 +1924,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D10">
-    <cfRule type="colorScale" priority="7">
+    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1802,7 +1936,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D11">
-    <cfRule type="colorScale" priority="2">
+    <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1810,6 +1944,146 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D12:D16">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:K5">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:K8 K12:K16">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:K16">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K6:K8">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K9">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K9:K10">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K10">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -1831,7 +2105,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D12:D15">
+  <conditionalFormatting sqref="K12:K16">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -1846,7 +2120,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="E3 E6 E9 E12 G6" formulaRange="1"/>
+    <ignoredError sqref="E3 E6 E9 G6 E12" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Mise à jour et en cohérence des livrets français et anglais
</commit_message>
<xml_diff>
--- a/docs/Cartes-Actions-Repartition.xlsx
+++ b/docs/Cartes-Actions-Repartition.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Documents\GitHub\Terre-de-Barons\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B62CBA3-942F-49DF-85E0-E00B635F0A7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4421B3C-404A-4126-B89B-AA674F338A99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-9120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -426,6 +426,56 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -443,9 +493,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -479,53 +526,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -836,12 +836,12 @@
       <c r="D2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="10"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="12"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="32"/>
       <c r="J2" s="3" t="s">
         <v>8</v>
       </c>
@@ -859,13 +859,13 @@
       <c r="D3" s="1">
         <v>4</v>
       </c>
-      <c r="E3" s="17">
+      <c r="E3" s="36">
         <f>SUM(D3:D5)</f>
         <v>15</v>
       </c>
-      <c r="F3" s="18"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="37">
+      <c r="F3" s="37"/>
+      <c r="G3" s="38"/>
+      <c r="H3" s="18">
         <f>SUM(D3:D16)</f>
         <v>43</v>
       </c>
@@ -886,10 +886,10 @@
       <c r="D4" s="1">
         <v>5</v>
       </c>
-      <c r="E4" s="20"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="38"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="19"/>
       <c r="J4" s="1" t="s">
         <v>12</v>
       </c>
@@ -907,10 +907,10 @@
       <c r="D5" s="1">
         <v>6</v>
       </c>
-      <c r="E5" s="23"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="38"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="19"/>
       <c r="J5" s="1" t="s">
         <v>13</v>
       </c>
@@ -928,19 +928,19 @@
       <c r="D6" s="2">
         <v>2</v>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="33">
         <f>SUM(D6:D8)</f>
         <v>9</v>
       </c>
-      <c r="F6" s="13">
+      <c r="F6" s="33">
         <f>E6+E9</f>
         <v>17</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="24">
         <f>SUM(D6:D11)</f>
         <v>23</v>
       </c>
-      <c r="H6" s="38"/>
+      <c r="H6" s="19"/>
       <c r="J6" s="2" t="s">
         <v>14</v>
       </c>
@@ -958,10 +958,10 @@
       <c r="D7" s="2">
         <v>3</v>
       </c>
-      <c r="E7" s="14"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="38"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="46"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="19"/>
       <c r="J7" s="2" t="s">
         <v>15</v>
       </c>
@@ -979,10 +979,10 @@
       <c r="D8" s="2">
         <v>4</v>
       </c>
-      <c r="E8" s="15"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="38"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="19"/>
       <c r="J8" s="2" t="s">
         <v>16</v>
       </c>
@@ -1000,13 +1000,13 @@
       <c r="D9" s="2">
         <v>3</v>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="33">
         <f>SUM(D9:D10)</f>
         <v>8</v>
       </c>
-      <c r="F9" s="27"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="38"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="19"/>
       <c r="J9" s="2" t="s">
         <v>2</v>
       </c>
@@ -1024,10 +1024,10 @@
       <c r="D10" s="2">
         <v>5</v>
       </c>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="38"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="45"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="19"/>
       <c r="J10" s="2" t="s">
         <v>1</v>
       </c>
@@ -1053,8 +1053,8 @@
         <f>E11</f>
         <v>6</v>
       </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="38"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="19"/>
       <c r="J11" s="2" t="s">
         <v>6</v>
       </c>
@@ -1072,13 +1072,13 @@
       <c r="D12" s="8">
         <v>1</v>
       </c>
-      <c r="E12" s="28">
+      <c r="E12" s="9">
         <f>SUM(D12:D16)</f>
         <v>5</v>
       </c>
-      <c r="F12" s="29"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="38"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="19"/>
       <c r="J12" s="1" t="s">
         <v>3</v>
       </c>
@@ -1096,10 +1096,10 @@
       <c r="D13" s="8">
         <v>1</v>
       </c>
-      <c r="E13" s="31"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="33"/>
-      <c r="H13" s="38"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="19"/>
       <c r="J13" s="1" t="s">
         <v>4</v>
       </c>
@@ -1117,10 +1117,10 @@
       <c r="D14" s="8">
         <v>1</v>
       </c>
-      <c r="E14" s="31"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="33"/>
-      <c r="H14" s="38"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="19"/>
       <c r="J14" s="1" t="s">
         <v>10</v>
       </c>
@@ -1138,10 +1138,10 @@
       <c r="D15" s="8">
         <v>1</v>
       </c>
-      <c r="E15" s="31"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="38"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="19"/>
       <c r="J15" s="5" t="s">
         <v>7</v>
       </c>
@@ -1159,10 +1159,10 @@
       <c r="D16" s="8">
         <v>1</v>
       </c>
-      <c r="E16" s="34"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="36"/>
-      <c r="H16" s="39"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="20"/>
       <c r="J16" s="5" t="s">
         <v>34</v>
       </c>
@@ -1493,12 +1493,12 @@
       <c r="D2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="40" t="s">
+      <c r="E2" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
       <c r="J2" s="6" t="s">
         <v>17</v>
       </c>
@@ -1516,13 +1516,13 @@
       <c r="D3" s="1">
         <v>4</v>
       </c>
-      <c r="E3" s="42">
+      <c r="E3" s="23">
         <f>SUM(D3:D5)</f>
         <v>15</v>
       </c>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="37">
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="18">
         <f>SUM(D3:D16)</f>
         <v>43</v>
       </c>
@@ -1543,10 +1543,10 @@
       <c r="D4" s="1">
         <v>5</v>
       </c>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="38"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="19"/>
       <c r="J4" s="1" t="s">
         <v>22</v>
       </c>
@@ -1564,10 +1564,10 @@
       <c r="D5" s="1">
         <v>6</v>
       </c>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="38"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="19"/>
       <c r="J5" s="1" t="s">
         <v>23</v>
       </c>
@@ -1585,19 +1585,19 @@
       <c r="D6" s="2">
         <v>2</v>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="24">
         <f>SUM(D6:D8)</f>
         <v>9</v>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="24">
         <f>E6+E9</f>
         <v>17</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="24">
         <f>SUM(D6:D11)</f>
         <v>23</v>
       </c>
-      <c r="H6" s="38"/>
+      <c r="H6" s="19"/>
       <c r="J6" s="2" t="s">
         <v>24</v>
       </c>
@@ -1615,10 +1615,10 @@
       <c r="D7" s="2">
         <v>3</v>
       </c>
-      <c r="E7" s="16"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="38"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="19"/>
       <c r="J7" s="2" t="s">
         <v>25</v>
       </c>
@@ -1636,10 +1636,10 @@
       <c r="D8" s="2">
         <v>4</v>
       </c>
-      <c r="E8" s="16"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="38"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="19"/>
       <c r="J8" s="2" t="s">
         <v>26</v>
       </c>
@@ -1657,13 +1657,13 @@
       <c r="D9" s="2">
         <v>3</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="24">
         <f>SUM(D9:D10)</f>
         <v>8</v>
       </c>
-      <c r="F9" s="43"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="38"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="19"/>
       <c r="J9" s="2" t="s">
         <v>27</v>
       </c>
@@ -1681,10 +1681,10 @@
       <c r="D10" s="2">
         <v>5</v>
       </c>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="38"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="19"/>
       <c r="J10" s="2" t="s">
         <v>28</v>
       </c>
@@ -1710,8 +1710,8 @@
         <f>E11</f>
         <v>6</v>
       </c>
-      <c r="G11" s="16"/>
-      <c r="H11" s="38"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="19"/>
       <c r="J11" s="2" t="s">
         <v>29</v>
       </c>
@@ -1729,13 +1729,13 @@
       <c r="D12" s="1">
         <v>1</v>
       </c>
-      <c r="E12" s="28">
+      <c r="E12" s="9">
         <f>SUM(D12:D16)</f>
         <v>5</v>
       </c>
-      <c r="F12" s="29"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="38"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="19"/>
       <c r="J12" s="1" t="s">
         <v>30</v>
       </c>
@@ -1753,10 +1753,10 @@
       <c r="D13" s="1">
         <v>1</v>
       </c>
-      <c r="E13" s="31"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="33"/>
-      <c r="H13" s="38"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="19"/>
       <c r="J13" s="1" t="s">
         <v>31</v>
       </c>
@@ -1774,10 +1774,10 @@
       <c r="D14" s="1">
         <v>1</v>
       </c>
-      <c r="E14" s="31"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="33"/>
-      <c r="H14" s="38"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="19"/>
       <c r="J14" s="1" t="s">
         <v>32</v>
       </c>
@@ -1795,10 +1795,10 @@
       <c r="D15" s="1">
         <v>1</v>
       </c>
-      <c r="E15" s="31"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="38"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="19"/>
       <c r="J15" s="5" t="s">
         <v>33</v>
       </c>
@@ -1816,10 +1816,10 @@
       <c r="D16" s="1">
         <v>1</v>
       </c>
-      <c r="E16" s="44"/>
-      <c r="F16" s="45"/>
-      <c r="G16" s="46"/>
-      <c r="H16" s="39"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="20"/>
       <c r="J16" s="5" t="s">
         <v>35</v>
       </c>

</xml_diff>